<commit_message>
updated guest list again
</commit_message>
<xml_diff>
--- a/my-wedding-site/data/Wedding planner - Guest list.xlsx
+++ b/my-wedding-site/data/Wedding planner - Guest list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Code\MarriageWebsite\my-wedding-site\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93FAEB6B-C646-4C0C-B025-9F3FBF5CBC9F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA3024A8-7DAF-48BC-A8B1-E7D044773E7C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guest list" sheetId="1" r:id="rId1"/>
@@ -265,12 +265,6 @@
     <t>Marsha +1</t>
   </si>
   <si>
-    <t>Matthew Ryan</t>
-  </si>
-  <si>
-    <t>Becca Ryan</t>
-  </si>
-  <si>
     <t>Lou Denaix</t>
   </si>
   <si>
@@ -329,6 +323,12 @@
   </si>
   <si>
     <t>Léon Jaubert</t>
+  </si>
+  <si>
+    <t>Matthew Bryan</t>
+  </si>
+  <si>
+    <t>Becca Bryan</t>
   </si>
 </sst>
 </file>
@@ -981,20 +981,20 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:P148"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="5.140625" customWidth="1"/>
-    <col min="2" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" customWidth="1"/>
-    <col min="6" max="7" width="14.140625" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" customWidth="1"/>
-    <col min="9" max="11" width="9.140625" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" customWidth="1"/>
-    <col min="13" max="13" width="8.42578125" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" customWidth="1"/>
-    <col min="15" max="15" width="17.7109375" customWidth="1"/>
-    <col min="16" max="16" width="5.140625" customWidth="1"/>
+    <col min="1" max="1" width="5.1796875" customWidth="1"/>
+    <col min="2" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" customWidth="1"/>
+    <col min="6" max="7" width="14.1796875" customWidth="1"/>
+    <col min="8" max="8" width="9.7265625" customWidth="1"/>
+    <col min="9" max="11" width="9.1796875" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" customWidth="1"/>
+    <col min="13" max="13" width="8.453125" customWidth="1"/>
+    <col min="14" max="14" width="14.26953125" customWidth="1"/>
+    <col min="15" max="15" width="17.7265625" customWidth="1"/>
+    <col min="16" max="16" width="5.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="6" customHeight="1">
@@ -2305,7 +2305,7 @@
         <v>30</v>
       </c>
       <c r="C61" s="26" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="D61" s="32"/>
       <c r="E61" s="27"/>
@@ -2325,7 +2325,7 @@
       <c r="A62" s="8"/>
       <c r="B62" s="18"/>
       <c r="C62" s="26" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D62" s="32"/>
       <c r="E62" s="27"/>
@@ -2347,7 +2347,7 @@
         <v>31</v>
       </c>
       <c r="C63" s="26" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D63" s="32"/>
       <c r="E63" s="27"/>
@@ -2367,7 +2367,7 @@
       <c r="A64" s="8"/>
       <c r="B64" s="18"/>
       <c r="C64" s="26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D64" s="32"/>
       <c r="E64" s="27"/>
@@ -2389,7 +2389,7 @@
         <v>32</v>
       </c>
       <c r="C65" s="26" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D65" s="32"/>
       <c r="E65" s="27"/>
@@ -2411,7 +2411,7 @@
         <v>33</v>
       </c>
       <c r="C66" s="26" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D66" s="32"/>
       <c r="E66" s="27"/>
@@ -2433,7 +2433,7 @@
         <v>34</v>
       </c>
       <c r="C67" s="26" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D67" s="32"/>
       <c r="E67" s="27"/>
@@ -2455,7 +2455,7 @@
         <v>35</v>
       </c>
       <c r="C68" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D68" s="32"/>
       <c r="E68" s="27"/>
@@ -2475,7 +2475,7 @@
       <c r="A69" s="8"/>
       <c r="B69" s="18"/>
       <c r="C69" s="26" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D69" s="32"/>
       <c r="E69" s="27"/>
@@ -2497,7 +2497,7 @@
         <v>36</v>
       </c>
       <c r="C70" s="26" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D70" s="32"/>
       <c r="E70" s="27"/>
@@ -2519,7 +2519,7 @@
         <v>37</v>
       </c>
       <c r="C71" s="26" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D71" s="32"/>
       <c r="E71" s="27"/>
@@ -2541,7 +2541,7 @@
         <v>38</v>
       </c>
       <c r="C72" s="26" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D72" s="32"/>
       <c r="E72" s="27"/>
@@ -2561,7 +2561,7 @@
       <c r="A73" s="8"/>
       <c r="B73" s="18"/>
       <c r="C73" s="26" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D73" s="32"/>
       <c r="E73" s="27"/>
@@ -2583,7 +2583,7 @@
         <v>39</v>
       </c>
       <c r="C74" s="26" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D74" s="32"/>
       <c r="E74" s="27"/>
@@ -2605,7 +2605,7 @@
         <v>40</v>
       </c>
       <c r="C75" s="26" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D75" s="32"/>
       <c r="E75" s="27"/>
@@ -2627,7 +2627,7 @@
         <v>41</v>
       </c>
       <c r="C76" s="34" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D76" s="32"/>
       <c r="E76" s="27"/>
@@ -2649,7 +2649,7 @@
         <v>42</v>
       </c>
       <c r="C77" s="26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D77" s="32"/>
       <c r="E77" s="27"/>
@@ -2671,7 +2671,7 @@
         <v>43</v>
       </c>
       <c r="C78" s="34" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D78" s="32"/>
       <c r="E78" s="27"/>
@@ -2693,7 +2693,7 @@
         <v>44</v>
       </c>
       <c r="C79" s="34" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D79" s="32"/>
       <c r="E79" s="27"/>
@@ -2715,7 +2715,7 @@
         <v>45</v>
       </c>
       <c r="C80" s="26" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D80" s="32"/>
       <c r="E80" s="27"/>
@@ -2735,7 +2735,7 @@
       <c r="A81" s="8"/>
       <c r="B81" s="18"/>
       <c r="C81" s="26" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D81" s="32"/>
       <c r="E81" s="27"/>
@@ -2755,7 +2755,7 @@
       <c r="A82" s="8"/>
       <c r="B82" s="37"/>
       <c r="C82" s="26" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D82" s="32"/>
       <c r="E82" s="27"/>

</xml_diff>